<commit_message>
se han corregido los errores identificados por los estudiantes
</commit_message>
<xml_diff>
--- a/data/key1/proyect2/files/Datum Corporation.xlsx
+++ b/data/key1/proyect2/files/Datum Corporation.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29530"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Teacher Sergio\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Teacher Sergio\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{4CCEC460-5E12-4112-A4F7-5DE49E75151E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3B677116-9292-40B3-BBD4-F55F531D6ACB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" activeTab="2" xr2:uid="{E8A519F3-2860-44F1-A7F2-CF0544AB9C00}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{E8A519F3-2860-44F1-A7F2-CF0544AB9C00}"/>
   </bookViews>
   <sheets>
     <sheet name="Orders" sheetId="2" r:id="rId1"/>
@@ -19,7 +19,7 @@
   </sheets>
   <calcPr calcId="191029"/>
   <pivotCaches>
-    <pivotCache cacheId="11" r:id="rId4"/>
+    <pivotCache cacheId="0" r:id="rId4"/>
   </pivotCaches>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -358,9 +358,9 @@
     <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="2" applyBorder="1" applyAlignment="1">
@@ -379,18 +379,17 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" pivotButton="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" indent="1"/>
+    </xf>
+    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" pivotButton="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Currency" xfId="1" builtinId="4"/>
@@ -398,35 +397,6 @@
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="17">
-    <dxf>
-      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="12" formatCode="&quot;$&quot;#,##0.00_);[Red]\(&quot;$&quot;#,##0.00\)"/>
-      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="12" formatCode="&quot;$&quot;#,##0.00_);[Red]\(&quot;$&quot;#,##0.00\)"/>
-      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
     <dxf>
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
@@ -463,6 +433,35 @@
     </dxf>
     <dxf>
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="12" formatCode="&quot;$&quot;#,##0.00_);[Red]\(&quot;$&quot;#,##0.00\)"/>
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="12" formatCode="&quot;$&quot;#,##0.00_);[Red]\(&quot;$&quot;#,##0.00\)"/>
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -781,7 +780,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{27488EE7-7194-4BED-BA03-FBACC9208520}" name="PivotTable2" cacheId="11" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{27488EE7-7194-4BED-BA03-FBACC9208520}" name="PivotTable2" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
   <location ref="A3:C20" firstHeaderRow="0" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="7">
     <pivotField showAll="0"/>
@@ -893,7 +892,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{93CF7390-95C9-4444-87CE-90384AA18A69}" name="Table2" displayName="Table2" ref="A3:G31" totalsRowShown="0" headerRowDxfId="1" dataDxfId="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{93CF7390-95C9-4444-87CE-90384AA18A69}" name="Table2" displayName="Table2" ref="A3:G31" totalsRowShown="0" headerRowDxfId="16" dataDxfId="15">
   <autoFilter ref="A3:G31" xr:uid="{93CF7390-95C9-4444-87CE-90384AA18A69}">
     <filterColumn colId="0" hiddenButton="1"/>
     <filterColumn colId="1" hiddenButton="1"/>
@@ -904,20 +903,20 @@
     <filterColumn colId="6" hiddenButton="1"/>
   </autoFilter>
   <tableColumns count="7">
-    <tableColumn id="1" xr3:uid="{67E6C122-BD05-4D00-A90A-FF25B23064F9}" name="Order ID" dataDxfId="8"/>
-    <tableColumn id="2" xr3:uid="{98FA0F1C-F1DF-4E39-AF88-1D5C49D76049}" name="Material" dataDxfId="7"/>
-    <tableColumn id="3" xr3:uid="{FDCE1D0B-AF9C-4C85-8F82-3B2FC3A4A01C}" name="Supplier" dataDxfId="6"/>
-    <tableColumn id="4" xr3:uid="{1B08D23E-6D84-4FC5-A7C9-82D34B7C13F2}" name="Unit size" dataDxfId="5"/>
-    <tableColumn id="5" xr3:uid="{928897BD-3AAC-4DF0-8E5E-9255C442D22F}" name="Unit Cost" dataDxfId="4"/>
-    <tableColumn id="6" xr3:uid="{B319D492-7F4F-4FD6-B98C-C564A5BDB178}" name="Quantity" dataDxfId="3"/>
-    <tableColumn id="7" xr3:uid="{D22FACBE-FC17-47EC-8CC8-52DA269EA9C7}" name="Order Total" dataDxfId="2"/>
+    <tableColumn id="1" xr3:uid="{67E6C122-BD05-4D00-A90A-FF25B23064F9}" name="Order ID" dataDxfId="14"/>
+    <tableColumn id="2" xr3:uid="{98FA0F1C-F1DF-4E39-AF88-1D5C49D76049}" name="Material" dataDxfId="13"/>
+    <tableColumn id="3" xr3:uid="{FDCE1D0B-AF9C-4C85-8F82-3B2FC3A4A01C}" name="Supplier" dataDxfId="12"/>
+    <tableColumn id="4" xr3:uid="{1B08D23E-6D84-4FC5-A7C9-82D34B7C13F2}" name="Unit size" dataDxfId="11"/>
+    <tableColumn id="5" xr3:uid="{928897BD-3AAC-4DF0-8E5E-9255C442D22F}" name="Unit Cost" dataDxfId="10"/>
+    <tableColumn id="6" xr3:uid="{B319D492-7F4F-4FD6-B98C-C564A5BDB178}" name="Quantity" dataDxfId="9"/>
+    <tableColumn id="7" xr3:uid="{D22FACBE-FC17-47EC-8CC8-52DA269EA9C7}" name="Order Total" dataDxfId="8"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight8" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{8A99BE9D-F60D-4A59-AE06-B7DB84A4E979}" name="Table1" displayName="Table1" ref="A1:E6" totalsRowShown="0" headerRowDxfId="16" dataDxfId="15" tableBorderDxfId="14">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{8A99BE9D-F60D-4A59-AE06-B7DB84A4E979}" name="Table1" displayName="Table1" ref="A1:E6" totalsRowShown="0" headerRowDxfId="7" dataDxfId="6" tableBorderDxfId="5">
   <autoFilter ref="A1:E6" xr:uid="{8A99BE9D-F60D-4A59-AE06-B7DB84A4E979}">
     <filterColumn colId="0" hiddenButton="1"/>
     <filterColumn colId="1" hiddenButton="1"/>
@@ -926,11 +925,11 @@
     <filterColumn colId="4" hiddenButton="1"/>
   </autoFilter>
   <tableColumns count="5">
-    <tableColumn id="1" xr3:uid="{314360B3-28A4-4D13-9139-5C44B55B7A24}" name="Supplier ID" dataDxfId="13"/>
-    <tableColumn id="2" xr3:uid="{52848A5A-EBEE-463C-8383-36251800CCBA}" name="Suppliers" dataDxfId="12"/>
-    <tableColumn id="3" xr3:uid="{3483A8F4-6AE4-4A59-9D66-9F4208EFBABC}" name="Contact" dataDxfId="11"/>
-    <tableColumn id="4" xr3:uid="{25EE7569-E6EE-4165-96A7-B97BA3DB8BBF}" name="Email Address" dataDxfId="10" dataCellStyle="Hyperlink"/>
-    <tableColumn id="5" xr3:uid="{80A328D1-B12B-4514-B879-EBB1A840CC47}" name="Telephone Number" dataDxfId="9"/>
+    <tableColumn id="1" xr3:uid="{314360B3-28A4-4D13-9139-5C44B55B7A24}" name="Supplier ID" dataDxfId="4"/>
+    <tableColumn id="2" xr3:uid="{52848A5A-EBEE-463C-8383-36251800CCBA}" name="Suppliers" dataDxfId="3"/>
+    <tableColumn id="3" xr3:uid="{3483A8F4-6AE4-4A59-9D66-9F4208EFBABC}" name="Contact" dataDxfId="2"/>
+    <tableColumn id="4" xr3:uid="{25EE7569-E6EE-4165-96A7-B97BA3DB8BBF}" name="Email Address" dataDxfId="1" dataCellStyle="Hyperlink"/>
+    <tableColumn id="5" xr3:uid="{80A328D1-B12B-4514-B879-EBB1A840CC47}" name="Telephone Number" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight8" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1256,10 +1255,10 @@
       <c r="A2" s="5" t="s">
         <v>26</v>
       </c>
-      <c r="I2" s="12" t="s">
+      <c r="I2" s="15" t="s">
         <v>44</v>
       </c>
-      <c r="J2" s="13"/>
+      <c r="J2" s="16"/>
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
@@ -1287,7 +1286,7 @@
         <v>29</v>
       </c>
       <c r="J3" s="10" t="s">
-        <v>7</v>
+        <v>51</v>
       </c>
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.25">
@@ -2095,7 +2094,7 @@
   </cols>
   <sheetData>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A3" s="14" t="s">
+      <c r="A3" s="12" t="s">
         <v>46</v>
       </c>
       <c r="B3" t="s">
@@ -2109,54 +2108,54 @@
       <c r="A4" s="3" t="s">
         <v>36</v>
       </c>
-      <c r="B4" s="16">
+      <c r="B4">
         <v>7</v>
       </c>
-      <c r="C4" s="17">
+      <c r="C4" s="14">
         <v>2816</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A5" s="15" t="s">
+      <c r="A5" s="13" t="s">
         <v>38</v>
       </c>
-      <c r="B5" s="16">
+      <c r="B5">
         <v>3</v>
       </c>
-      <c r="C5" s="17">
+      <c r="C5" s="14">
         <v>1020</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A6" s="15" t="s">
+      <c r="A6" s="13" t="s">
         <v>50</v>
       </c>
-      <c r="B6" s="16">
+      <c r="B6">
         <v>2</v>
       </c>
-      <c r="C6" s="17">
+      <c r="C6" s="14">
         <v>996</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A7" s="15" t="s">
+      <c r="A7" s="13" t="s">
         <v>51</v>
       </c>
-      <c r="B7" s="16">
+      <c r="B7">
         <v>1</v>
       </c>
-      <c r="C7" s="17">
+      <c r="C7" s="14">
         <v>500</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A8" s="15" t="s">
+      <c r="A8" s="13" t="s">
         <v>9</v>
       </c>
-      <c r="B8" s="16">
+      <c r="B8">
         <v>1</v>
       </c>
-      <c r="C8" s="17">
+      <c r="C8" s="14">
         <v>300</v>
       </c>
     </row>
@@ -2164,43 +2163,43 @@
       <c r="A9" s="3" t="s">
         <v>34</v>
       </c>
-      <c r="B9" s="16">
+      <c r="B9">
         <v>8</v>
       </c>
-      <c r="C9" s="17">
+      <c r="C9" s="14">
         <v>1838.75</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A10" s="15" t="s">
+      <c r="A10" s="13" t="s">
         <v>38</v>
       </c>
-      <c r="B10" s="16">
+      <c r="B10">
         <v>4</v>
       </c>
-      <c r="C10" s="17">
+      <c r="C10" s="14">
         <v>906.75</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A11" s="15" t="s">
+      <c r="A11" s="13" t="s">
         <v>50</v>
       </c>
-      <c r="B11" s="16">
+      <c r="B11">
         <v>3</v>
       </c>
-      <c r="C11" s="17">
+      <c r="C11" s="14">
         <v>792</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A12" s="15" t="s">
+      <c r="A12" s="13" t="s">
         <v>9</v>
       </c>
-      <c r="B12" s="16">
+      <c r="B12">
         <v>1</v>
       </c>
-      <c r="C12" s="17">
+      <c r="C12" s="14">
         <v>140</v>
       </c>
     </row>
@@ -2208,32 +2207,32 @@
       <c r="A13" s="3" t="s">
         <v>37</v>
       </c>
-      <c r="B13" s="16">
+      <c r="B13">
         <v>6</v>
       </c>
-      <c r="C13" s="17">
+      <c r="C13" s="14">
         <v>707.5</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A14" s="15" t="s">
+      <c r="A14" s="13" t="s">
         <v>38</v>
       </c>
-      <c r="B14" s="16">
+      <c r="B14">
         <v>5</v>
       </c>
-      <c r="C14" s="17">
+      <c r="C14" s="14">
         <v>570</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A15" s="15" t="s">
+      <c r="A15" s="13" t="s">
         <v>51</v>
       </c>
-      <c r="B15" s="16">
+      <c r="B15">
         <v>1</v>
       </c>
-      <c r="C15" s="17">
+      <c r="C15" s="14">
         <v>137.5</v>
       </c>
     </row>
@@ -2241,43 +2240,43 @@
       <c r="A16" s="3" t="s">
         <v>35</v>
       </c>
-      <c r="B16" s="16">
+      <c r="B16">
         <v>7</v>
       </c>
-      <c r="C16" s="17">
+      <c r="C16" s="14">
         <v>1961.5</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A17" s="15" t="s">
+      <c r="A17" s="13" t="s">
         <v>38</v>
       </c>
-      <c r="B17" s="16">
+      <c r="B17">
         <v>4</v>
       </c>
-      <c r="C17" s="17">
+      <c r="C17" s="14">
         <v>1139.5</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A18" s="15" t="s">
+      <c r="A18" s="13" t="s">
         <v>51</v>
       </c>
-      <c r="B18" s="16">
+      <c r="B18">
         <v>1</v>
       </c>
-      <c r="C18" s="17">
+      <c r="C18" s="14">
         <v>240</v>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A19" s="15" t="s">
+      <c r="A19" s="13" t="s">
         <v>9</v>
       </c>
-      <c r="B19" s="16">
+      <c r="B19">
         <v>2</v>
       </c>
-      <c r="C19" s="17">
+      <c r="C19" s="14">
         <v>582</v>
       </c>
     </row>
@@ -2285,10 +2284,10 @@
       <c r="A20" s="3" t="s">
         <v>47</v>
       </c>
-      <c r="B20" s="16">
+      <c r="B20">
         <v>28</v>
       </c>
-      <c r="C20" s="17">
+      <c r="C20" s="14">
         <v>7323.75</v>
       </c>
     </row>

</xml_diff>